<commit_message>
Accumulated updates and oneoffs cleanup
- Remove completed oneoffs scripts (70+ files)
- Update shared modules (api-client, notifier, franchise-api, etc.)
- Update LAM workflow scripts and data files
- Update documentation (roadmaps, workflow docs)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM EPG Award/Lam_EPG_SIPOC.xlsx
+++ b/Trading Analysis/LAM EPG Award/Lam_EPG_SIPOC.xlsx
@@ -1605,6 +1605,9 @@
       <c r="AA14" t="str">
         <v>POV0075267</v>
       </c>
+      <c r="AI14" t="str">
+        <v>380734306742</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -2894,6 +2897,9 @@
       <c r="AA31" t="str">
         <v>POV0075267</v>
       </c>
+      <c r="AI31" t="str">
+        <v>380734306742</v>
+      </c>
     </row>
     <row r="32" xml:space="preserve">
       <c r="A32" t="str">
@@ -3141,6 +3147,9 @@
       <c r="AA34" t="str">
         <v>POV0075267</v>
       </c>
+      <c r="AI34" t="str">
+        <v>380734306742</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -4887,6 +4896,9 @@
       <c r="AA56" t="str">
         <v>POV0075267</v>
       </c>
+      <c r="AI56" t="str">
+        <v>380734306742</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -7580,6 +7592,9 @@
       <c r="AA88" t="str">
         <v>POV0075267</v>
       </c>
+      <c r="AI88" t="str">
+        <v>380734306742</v>
+      </c>
     </row>
     <row r="89" xml:space="preserve">
       <c r="A89" t="str">
@@ -7804,6 +7819,9 @@
       <c r="AA91" t="str">
         <v>POV0075267</v>
       </c>
+      <c r="AI91" t="str">
+        <v>380734306742</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -11111,6 +11129,9 @@
       <c r="AA133" t="str">
         <v>POV0075267</v>
       </c>
+      <c r="AI133" t="str">
+        <v>380734306742</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -11543,8 +11564,29 @@
       <c r="M139">
         <v>15.514632</v>
       </c>
+      <c r="P139" t="str">
+        <v>Mouser</v>
+      </c>
+      <c r="R139">
+        <v>15</v>
+      </c>
+      <c r="AA139" t="str">
+        <v>POV0075856</v>
+      </c>
+      <c r="AB139" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="AF139" t="str">
+        <v>PO809925</v>
+      </c>
       <c r="AH139" t="str">
         <v>DigiKey stock $15.41 (over base $17.72 — under); Newark stock $17.92 (over base). Try DigiKey first; if restricted then Newark; if that fails Amalfi</v>
+      </c>
+      <c r="AI139" t="str">
+        <v>528979457439</v>
+      </c>
+      <c r="AJ139" t="str">
+        <v>Y</v>
       </c>
     </row>
     <row r="140">
@@ -11597,10 +11639,10 @@
         <v>Mouser</v>
       </c>
       <c r="Q140">
-        <v>8.75</v>
+        <v>15</v>
       </c>
       <c r="R140">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="S140">
         <v>0</v>
@@ -11615,10 +11657,19 @@
         <v>-40.70500000000001</v>
       </c>
       <c r="AA140" t="str">
-        <v>POV0075257</v>
+        <v>POV0075856</v>
+      </c>
+      <c r="AB140" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="AF140" t="str">
+        <v>PO809925</v>
       </c>
       <c r="AI140" t="str">
-        <v>518989245440 shipped 03/26</v>
+        <v>528979457439</v>
+      </c>
+      <c r="AJ140" t="str">
+        <v>Y</v>
       </c>
     </row>
     <row r="141">

</xml_diff>